<commit_message>
Strengthen risk report with date audit and review economics
</commit_message>
<xml_diff>
--- a/fintechathon-topic3/outputs/分析结果汇总.xlsx
+++ b/fintechathon-topic3/outputs/分析结果汇总.xlsx
@@ -1,25 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="阅读说明" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="指标说明" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="描述分析" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="模型比较" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="复核预算" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="敏感性检查" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="主模型置换重要性" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="主模型回归系数" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="模型置信区间" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="数据审计" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="阅读说明" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="指标说明" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="描述分析" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="模型比较" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="复核预算" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="敏感性检查" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="主模型置换重要性" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="主模型回归系数" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追加日期审计" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="模型置信区间" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据审计" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'阅读说明'!$A$1:$A$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'阅读说明'!$A$1:$A$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'指标说明'!$A$1:$E$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'描述分析'!$A$1:$K$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'模型比较'!$A$1:$J$7</definedName>
@@ -27,8 +28,9 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'敏感性检查'!$A$1:$F$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'主模型置换重要性'!$A$1:$D$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'主模型回归系数'!$A$1:$B$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'模型置信区间'!$A$1:$D$31</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'数据审计'!$A$1:$B$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'追加日期审计'!$A$1:$G$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'模型置信区间'!$A$1:$D$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'数据审计'!$A$1:$B$20</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -433,10 +435,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="45" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -502,13 +504,603 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>追加日期审计在原测试结果之后设计，不调参，不作为确认性检验；2017子组只有2家停业。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:A9"/>
+  <autoFilter ref="A1:A10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D31"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="21" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>model</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>metric</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>lower95</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>upper95</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>LR_Q</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>roc_auc</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>0.4256713707032275</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.6677424263553036</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>LR_Q</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>pr_auc_ap</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>0.1356471034841732</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.3567142380444</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>LR_Q</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>precision10</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.4285714285714285</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>LR_Q</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>recall10</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.2272727272727273</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>LR_Q</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>lift10</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" t="n">
+        <v>2.191558441558441</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>LR_QA</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>roc_auc</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>0.4298706352133772</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.675756599963659</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>LR_QA</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>pr_auc_ap</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>0.1390334860108768</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.3538441103911809</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>LR_QA</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>precision10</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.4285714285714285</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>LR_QA</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>recall10</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>LR_QA</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>lift10</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" t="n">
+        <v>2.410714285714286</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>LR_QAT</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>roc_auc</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>0.4539636363636364</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0.7016636363636362</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>LR_QAT</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>pr_auc_ap</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>0.1460729249758087</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0.3543375757424704</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>LR_QAT</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>precision10</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0.4285714285714285</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>LR_QAT</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>recall10</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0.2272727272727273</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>LR_QAT</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>lift10</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" t="n">
+        <v>2.191558441558441</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>HGB_Q</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>roc_auc</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>0.4487623546503791</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0.7173308611201917</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>HGB_Q</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>pr_auc_ap</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>0.162296408674153</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0.4177118672864044</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>HGB_Q</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>precision10</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>0.07142857142857142</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0.5714285714285714</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>HGB_Q</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>recall10</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>0.05263157894736842</v>
+      </c>
+      <c r="D20" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>HGB_Q</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>lift10</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>0.5075187969924811</v>
+      </c>
+      <c r="D21" t="n">
+        <v>3.214285714285714</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>HGB_QA</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>roc_auc</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>0.4890134553231071</v>
+      </c>
+      <c r="D22" t="n">
+        <v>0.7325218500797448</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>HGB_QA</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>pr_auc_ap</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>0.1786970943784346</v>
+      </c>
+      <c r="D23" t="n">
+        <v>0.4844062254239541</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>HGB_QA</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>precision10</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>0.07142857142857142</v>
+      </c>
+      <c r="D24" t="n">
+        <v>0.5714285714285714</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>HGB_QA</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>recall10</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>0.05967023172905526</v>
+      </c>
+      <c r="D25" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>HGB_QA</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>lift10</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>0.5753915202444614</v>
+      </c>
+      <c r="D26" t="n">
+        <v>3.214285714285714</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>HGB_QAT</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>roc_auc</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>0.5046607795901782</v>
+      </c>
+      <c r="D27" t="n">
+        <v>0.7515075338604751</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>HGB_QAT</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>pr_auc_ap</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>0.1992497107281067</v>
+      </c>
+      <c r="D28" t="n">
+        <v>0.5213186838346856</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>HGB_QAT</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>precision10</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>0.1428571428571428</v>
+      </c>
+      <c r="D29" t="n">
+        <v>0.7142857142857143</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>HGB_QAT</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>recall10</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D30" t="n">
+        <v>0.3888888888888889</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>HGB_QAT</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>lift10</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>0.9642857142857143</v>
+      </c>
+      <c r="D31" t="n">
+        <v>3.75</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:D31"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3174,13 +3766,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D31"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3191,17 +3786,32 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>metric</t>
+          <t>subset</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>lower95</t>
+          <t>merchants</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>upper95</t>
+          <t>closed</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>prevalence</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>roc_auc</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>ap</t>
         </is>
       </c>
     </row>
@@ -3213,14 +3823,23 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>roc_auc</t>
+          <t>all_test</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.4256713707032275</v>
+        <v>135</v>
       </c>
       <c r="D2" t="n">
-        <v>0.6677424263553036</v>
+        <v>25</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.1851851851851851</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.5447272727272727</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.2110153550488432</v>
       </c>
     </row>
     <row r="3">
@@ -3231,14 +3850,23 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>pr_auc_ap</t>
+          <t>year_2017</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.1356471034841732</v>
+        <v>107</v>
       </c>
       <c r="D3" t="n">
-        <v>0.3567142380444</v>
+        <v>2</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.0186915887850467</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.6857142857142857</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.0429292929292929</v>
       </c>
     </row>
     <row r="4">
@@ -3249,50 +3877,75 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>precision10</t>
+          <t>same_year_pairs</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0</v>
+        <v>135</v>
       </c>
       <c r="D4" t="n">
-        <v>0.4285714285714285</v>
-      </c>
+        <v>25</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.1851851851851851</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.6288461538461538</v>
+      </c>
+      <c r="G4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>LR_Q</t>
+          <t>LR_QA</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>recall10</t>
+          <t>all_test</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0</v>
+        <v>135</v>
       </c>
       <c r="D5" t="n">
-        <v>0.2272727272727273</v>
+        <v>25</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.1851851851851851</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.552</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.2123204177611183</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>LR_Q</t>
+          <t>LR_QA</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>lift10</t>
+          <t>year_2017</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0</v>
+        <v>107</v>
       </c>
       <c r="D6" t="n">
-        <v>2.191558441558441</v>
+        <v>2</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.0186915887850467</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.7142857142857142</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.0464743589743589</v>
       </c>
     </row>
     <row r="7">
@@ -3303,450 +3956,341 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>roc_auc</t>
+          <t>same_year_pairs</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.4298706352133772</v>
+        <v>135</v>
       </c>
       <c r="D7" t="n">
-        <v>0.675756599963659</v>
-      </c>
+        <v>25</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.1851851851851851</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.6653846153846154</v>
+      </c>
+      <c r="G7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>LR_QA</t>
+          <t>LR_QAT</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>pr_auc_ap</t>
+          <t>all_test</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.1390334860108768</v>
+        <v>135</v>
       </c>
       <c r="D8" t="n">
-        <v>0.3538441103911809</v>
+        <v>25</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.1851851851851851</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.5770909090909091</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.2200867440559849</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>LR_QA</t>
+          <t>LR_QAT</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>precision10</t>
+          <t>year_2017</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0</v>
+        <v>107</v>
       </c>
       <c r="D9" t="n">
-        <v>0.4285714285714285</v>
+        <v>2</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.0186915887850467</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.7380952380952381</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.0502450980392156</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>LR_QA</t>
+          <t>LR_QAT</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>recall10</t>
+          <t>same_year_pairs</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0</v>
+        <v>135</v>
       </c>
       <c r="D10" t="n">
-        <v>0.25</v>
-      </c>
+        <v>25</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.1851851851851851</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.6730769230769231</v>
+      </c>
+      <c r="G10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>LR_QA</t>
+          <t>HGB_Q</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>lift10</t>
+          <t>all_test</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0</v>
+        <v>135</v>
       </c>
       <c r="D11" t="n">
-        <v>2.410714285714286</v>
+        <v>25</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.1851851851851851</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.5845454545454545</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.2534682942887792</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>LR_QAT</t>
+          <t>HGB_Q</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>roc_auc</t>
+          <t>year_2017</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0.4539636363636364</v>
+        <v>107</v>
       </c>
       <c r="D12" t="n">
-        <v>0.7016636363636362</v>
+        <v>2</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0.0186915887850467</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0.5952380952380952</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0.0349119611414693</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>LR_QAT</t>
+          <t>HGB_Q</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>pr_auc_ap</t>
+          <t>same_year_pairs</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>0.1460729249758087</v>
+        <v>135</v>
       </c>
       <c r="D13" t="n">
-        <v>0.3543375757424704</v>
-      </c>
+        <v>25</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0.1851851851851851</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0.5557692307692308</v>
+      </c>
+      <c r="G13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>LR_QAT</t>
+          <t>HGB_QA</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>precision10</t>
+          <t>all_test</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0</v>
+        <v>135</v>
       </c>
       <c r="D14" t="n">
-        <v>0.4285714285714285</v>
+        <v>25</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0.1851851851851851</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0.6138181818181818</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0.2994156844861536</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>LR_QAT</t>
+          <t>HGB_QA</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>recall10</t>
+          <t>year_2017</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0</v>
+        <v>107</v>
       </c>
       <c r="D15" t="n">
-        <v>0.2272727272727273</v>
+        <v>2</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0.0186915887850467</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0.5714285714285714</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0.0328663793103448</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>LR_QAT</t>
+          <t>HGB_QA</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>lift10</t>
+          <t>same_year_pairs</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>0</v>
+        <v>135</v>
       </c>
       <c r="D16" t="n">
-        <v>2.191558441558441</v>
-      </c>
+        <v>25</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0.1851851851851851</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0.5653846153846154</v>
+      </c>
+      <c r="G16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>HGB_Q</t>
+          <t>HGB_QAT</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>roc_auc</t>
+          <t>all_test</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>0.4487623546503791</v>
+        <v>135</v>
       </c>
       <c r="D17" t="n">
-        <v>0.7173308611201917</v>
+        <v>25</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0.1851851851851851</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0.6309090909090909</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0.319234347720385</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>HGB_Q</t>
+          <t>HGB_QAT</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>pr_auc_ap</t>
+          <t>year_2017</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>0.162296408674153</v>
+        <v>107</v>
       </c>
       <c r="D18" t="n">
-        <v>0.4177118672864044</v>
+        <v>2</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0.0186915887850467</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0.4809523809523809</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0.0416666666666666</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>HGB_Q</t>
+          <t>HGB_QAT</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>precision10</t>
+          <t>same_year_pairs</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>0.07142857142857142</v>
+        <v>135</v>
       </c>
       <c r="D19" t="n">
-        <v>0.5714285714285714</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>HGB_Q</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>recall10</t>
-        </is>
-      </c>
-      <c r="C20" t="n">
-        <v>0.05263157894736842</v>
-      </c>
-      <c r="D20" t="n">
-        <v>0.3333333333333333</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>HGB_Q</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>lift10</t>
-        </is>
-      </c>
-      <c r="C21" t="n">
-        <v>0.5075187969924811</v>
-      </c>
-      <c r="D21" t="n">
-        <v>3.214285714285714</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>HGB_QA</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>roc_auc</t>
-        </is>
-      </c>
-      <c r="C22" t="n">
-        <v>0.4890134553231071</v>
-      </c>
-      <c r="D22" t="n">
-        <v>0.7325218500797448</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>HGB_QA</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>pr_auc_ap</t>
-        </is>
-      </c>
-      <c r="C23" t="n">
-        <v>0.1786970943784346</v>
-      </c>
-      <c r="D23" t="n">
-        <v>0.4844062254239541</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>HGB_QA</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>precision10</t>
-        </is>
-      </c>
-      <c r="C24" t="n">
-        <v>0.07142857142857142</v>
-      </c>
-      <c r="D24" t="n">
-        <v>0.5714285714285714</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>HGB_QA</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>recall10</t>
-        </is>
-      </c>
-      <c r="C25" t="n">
-        <v>0.05967023172905526</v>
-      </c>
-      <c r="D25" t="n">
-        <v>0.3333333333333333</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>HGB_QA</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>lift10</t>
-        </is>
-      </c>
-      <c r="C26" t="n">
-        <v>0.5753915202444614</v>
-      </c>
-      <c r="D26" t="n">
-        <v>3.214285714285714</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>HGB_QAT</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>roc_auc</t>
-        </is>
-      </c>
-      <c r="C27" t="n">
-        <v>0.5046607795901782</v>
-      </c>
-      <c r="D27" t="n">
-        <v>0.7515075338604751</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>HGB_QAT</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>pr_auc_ap</t>
-        </is>
-      </c>
-      <c r="C28" t="n">
-        <v>0.1992497107281067</v>
-      </c>
-      <c r="D28" t="n">
-        <v>0.5213186838346856</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>HGB_QAT</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>precision10</t>
-        </is>
-      </c>
-      <c r="C29" t="n">
-        <v>0.1428571428571428</v>
-      </c>
-      <c r="D29" t="n">
-        <v>0.7142857142857143</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>HGB_QAT</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>recall10</t>
-        </is>
-      </c>
-      <c r="C30" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="D30" t="n">
-        <v>0.3888888888888889</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>HGB_QAT</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>lift10</t>
-        </is>
-      </c>
-      <c r="C31" t="n">
-        <v>0.9642857142857143</v>
-      </c>
-      <c r="D31" t="n">
-        <v>3.75</v>
-      </c>
+        <v>25</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0.1851851851851851</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0.4884615384615384</v>
+      </c>
+      <c r="G19" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D31"/>
+  <autoFilter ref="A1:G19"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Complete evidence-to-decision report and prospective validation loop
</commit_message>
<xml_diff>
--- a/fintechathon-topic3/outputs/分析结果汇总.xlsx
+++ b/fintechathon-topic3/outputs/分析结果汇总.xlsx
@@ -16,8 +16,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="主模型置换重要性" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="主模型回归系数" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追加日期审计" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="模型置信区间" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据审计" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="概率评分审计" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="指标相关性" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="模型置信区间" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据审计" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'阅读说明'!$A$1:$A$10</definedName>
@@ -29,8 +31,10 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'主模型置换重要性'!$A$1:$D$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'主模型回归系数'!$A$1:$B$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'追加日期审计'!$A$1:$G$19</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'模型置信区间'!$A$1:$D$31</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'数据审计'!$A$1:$B$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'概率评分审计'!$A$1:$B$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'指标相关性'!$A$1:$D$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'模型置信区间'!$A$1:$D$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'数据审计'!$A$1:$B$20</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -523,6 +527,146 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>model</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>brier</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>fitting_prevalence_constant</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>0.1509029690847873</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>LR_QAT</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0.1662650743094656</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>HGB_QAT</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0.151877512528309</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:B4"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>feature_a</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>feature_b</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>spearman</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>fitting_merchants</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>rating_mean_360</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>low_rating_share_360</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>-0.9335334489917808</v>
+      </c>
+      <c r="D2" t="n">
+        <v>539</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>recent_reviews_180</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>previous_reviews_180</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>0.7359314644423012</v>
+      </c>
+      <c r="D3" t="n">
+        <v>539</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:D3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1100,7 +1244,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1372,7 +1516,7 @@
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="65" customWidth="1" min="3" max="3"/>
     <col width="80" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="33" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1490,7 +1634,7 @@
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>训练集拟合中位数填补</t>
+          <t>拟合数据中位数填补并加缺失指示；调参仅训练集，最终训练+验证集</t>
         </is>
       </c>
     </row>

</xml_diff>